<commit_message>
EPBDS-16837 Keep int[] in array functions and fix remove failing on a null array
sort, slice, remove, removeElement and removeNulls return the type of the array;
add, addAll and addElement widen it only to fit an added element.
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/7-Functions/ArrayFunctions.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/7-Functions/ArrayFunctions.xlsx
@@ -550,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I106"/>
+  <dimension ref="B2:I126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -1445,10 +1445,10 @@
       </c>
       <c r="D74" s="10" t="n"/>
     </row>
-    <row r="76" ht="16.5" customHeight="1">
+    <row r="76" ht="30" customHeight="1">
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>The functions keep the element type: applied to an array of a datatype, they return an array of the same datatype, so a field of an element is read directly without a cast.</t>
+          <t>The functions keep the element type: applied to an array of a datatype, they return an array of the same datatype, so a field of an element is read directly without a cast. A primitive array, such as int[], stays int[]. add, addAll and addElement change the type only to fit an added element: an Integer gives Integer[], so that the element can be empty, and a fraction gives double[].</t>
         </is>
       </c>
     </row>
@@ -1650,130 +1650,420 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>NumbersSorted</t>
+        </is>
+      </c>
+      <c r="C98" s="7" t="inlineStr">
+        <is>
+          <t>= sort(new int[] {3, 1, 2}).getClass().getSimpleName()</t>
+        </is>
+      </c>
+    </row>
     <row r="99">
-      <c r="B99" s="3" t="inlineStr">
+      <c r="B99" s="6" t="inlineStr">
+        <is>
+          <t>NumbersSliced</t>
+        </is>
+      </c>
+      <c r="C99" s="7" t="inlineStr">
+        <is>
+          <t>= slice(new int[] {1, 2, 3}, 1).getClass().getSimpleName()</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>NumbersRemoved</t>
+        </is>
+      </c>
+      <c r="C100" s="7" t="inlineStr">
+        <is>
+          <t>= remove(new int[] {1, 2}, 0).getClass().getSimpleName()</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>NumbersRemovedElement</t>
+        </is>
+      </c>
+      <c r="C101" s="7" t="inlineStr">
+        <is>
+          <t>= removeElement(new int[] {1, 2}, 1).getClass().getSimpleName()</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="B102" s="6" t="inlineStr">
+        <is>
+          <t>NumbersWithoutNulls</t>
+        </is>
+      </c>
+      <c r="C102" s="7" t="inlineStr">
+        <is>
+          <t>= removeNulls(new int[] {1, 2}).getClass().getSimpleName()</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="B103" s="6" t="inlineStr">
+        <is>
+          <t>NumbersInserted</t>
+        </is>
+      </c>
+      <c r="C103" s="7" t="inlineStr">
+        <is>
+          <t>= addElement(new int[] {1, 2}, 1, 5).getClass().getSimpleName()</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="B104" s="6" t="inlineStr">
+        <is>
+          <t>NumbersAdded</t>
+        </is>
+      </c>
+      <c r="C104" s="7" t="inlineStr">
+        <is>
+          <t>= add(new int[] {1, 2}, 3).getClass().getSimpleName()</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="B105" s="6" t="inlineStr">
+        <is>
+          <t>NumbersWithEmpty</t>
+        </is>
+      </c>
+      <c r="C105" s="7" t="inlineStr">
+        <is>
+          <t>= add(new int[] {1, 2}, (Integer) null).getClass().getSimpleName()</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="B106" s="6" t="inlineStr">
+        <is>
+          <t>NumbersWithFraction</t>
+        </is>
+      </c>
+      <c r="C106" s="7" t="inlineStr">
+        <is>
+          <t>= add(new int[] {1, 2}, 2.5).getClass().getSimpleName()</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="B107" s="6" t="inlineStr">
+        <is>
+          <t>FractionAdded</t>
+        </is>
+      </c>
+      <c r="C107" s="7" t="inlineStr">
+        <is>
+          <t>= add(new int[] {1, 2}, 2.5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="B109" s="3" t="inlineStr">
         <is>
           <t>Test TypedResults TypedResultsTest</t>
         </is>
       </c>
-      <c r="C99" s="8" t="n"/>
-      <c r="D99" s="4" t="n"/>
-    </row>
-    <row r="100">
-      <c r="B100" s="9" t="inlineStr">
+      <c r="C109" s="8" t="n"/>
+      <c r="D109" s="4" t="n"/>
+    </row>
+    <row r="110">
+      <c r="B110" s="9" t="inlineStr">
         <is>
           <t>_res_.$Added</t>
         </is>
       </c>
-      <c r="C100" s="5" t="inlineStr">
+      <c r="C110" s="5" t="inlineStr">
         <is>
           <t>add(countries, new Country(name = "Denmark"))[3].name</t>
         </is>
       </c>
-      <c r="D100" s="10" t="inlineStr">
+      <c r="D110" s="10" t="inlineStr">
         <is>
           <t>Denmark</t>
         </is>
       </c>
     </row>
-    <row r="101">
-      <c r="B101" s="9" t="inlineStr">
+    <row r="111">
+      <c r="B111" s="9" t="inlineStr">
         <is>
           <t>_res_.$AddedNames</t>
         </is>
       </c>
-      <c r="C101" s="5" t="inlineStr">
+      <c r="C111" s="5" t="inlineStr">
         <is>
           <t>add(countries, new Country(name = "Denmark")).name</t>
         </is>
       </c>
-      <c r="D101" s="10" t="inlineStr">
+      <c r="D111" s="10" t="inlineStr">
         <is>
           <t>Austria, Brazil, Chile, Denmark</t>
         </is>
       </c>
     </row>
-    <row r="102">
-      <c r="B102" s="9" t="inlineStr">
+    <row r="112">
+      <c r="B112" s="9" t="inlineStr">
         <is>
           <t>_res_.$AddedAll</t>
         </is>
       </c>
-      <c r="C102" s="5" t="inlineStr">
+      <c r="C112" s="5" t="inlineStr">
         <is>
           <t>addAll(countries, countries)[4].name</t>
         </is>
       </c>
-      <c r="D102" s="10" t="inlineStr">
+      <c r="D112" s="10" t="inlineStr">
         <is>
           <t>Brazil</t>
         </is>
       </c>
     </row>
-    <row r="103">
-      <c r="B103" s="9" t="inlineStr">
+    <row r="113">
+      <c r="B113" s="9" t="inlineStr">
         <is>
           <t>_res_.$Inserted</t>
         </is>
       </c>
-      <c r="C103" s="5" t="inlineStr">
+      <c r="C113" s="5" t="inlineStr">
         <is>
           <t>addElement(countries, 1, new Country(name = "Denmark"))[1].name</t>
         </is>
       </c>
-      <c r="D103" s="10" t="inlineStr">
+      <c r="D113" s="10" t="inlineStr">
         <is>
           <t>Denmark</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="B104" s="9" t="inlineStr">
+    <row r="114">
+      <c r="B114" s="9" t="inlineStr">
         <is>
           <t>_res_.$Removed</t>
         </is>
       </c>
-      <c r="C104" s="5" t="inlineStr">
+      <c r="C114" s="5" t="inlineStr">
         <is>
           <t>remove(countries, 0)[0].name</t>
         </is>
       </c>
-      <c r="D104" s="10" t="inlineStr">
+      <c r="D114" s="10" t="inlineStr">
         <is>
           <t>Brazil</t>
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="B105" s="9" t="inlineStr">
+    <row r="115">
+      <c r="B115" s="9" t="inlineStr">
         <is>
           <t>_res_.$RemovedElement</t>
         </is>
       </c>
-      <c r="C105" s="5" t="inlineStr">
+      <c r="C115" s="5" t="inlineStr">
         <is>
           <t>removeElement(countries, countries[1]).name</t>
         </is>
       </c>
-      <c r="D105" s="10" t="inlineStr">
+      <c r="D115" s="10" t="inlineStr">
         <is>
           <t>Austria, Chile</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="B106" s="9" t="inlineStr">
+    <row r="116">
+      <c r="B116" s="9" t="inlineStr">
         <is>
           <t>_res_.$WithoutNulls</t>
         </is>
       </c>
-      <c r="C106" s="5" t="inlineStr">
+      <c r="C116" s="5" t="inlineStr">
         <is>
           <t>removeNulls(new Country[] {null, countries[2]})[0].code</t>
         </is>
       </c>
-      <c r="D106" s="10" t="n">
+      <c r="D116" s="10" t="n">
         <v>56</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="B117" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NumbersSorted</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>sort(new int[] {3, 1, 2}).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D117" s="10" t="inlineStr">
+        <is>
+          <t>int[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="B118" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NumbersSliced</t>
+        </is>
+      </c>
+      <c r="C118" s="5" t="inlineStr">
+        <is>
+          <t>slice(new int[] {1, 2, 3}, 1).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D118" s="10" t="inlineStr">
+        <is>
+          <t>int[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="B119" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NumbersRemoved</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>remove(new int[] {1, 2}, 0).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D119" s="10" t="inlineStr">
+        <is>
+          <t>int[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="B120" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NumbersRemovedElement</t>
+        </is>
+      </c>
+      <c r="C120" s="5" t="inlineStr">
+        <is>
+          <t>removeElement(new int[] {1, 2}, 1).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D120" s="10" t="inlineStr">
+        <is>
+          <t>int[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="B121" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NumbersWithoutNulls</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>removeNulls(new int[] {1, 2}).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D121" s="10" t="inlineStr">
+        <is>
+          <t>int[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="B122" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NumbersInserted</t>
+        </is>
+      </c>
+      <c r="C122" s="5" t="inlineStr">
+        <is>
+          <t>addElement(new int[] {1, 2}, 1, 5).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D122" s="10" t="inlineStr">
+        <is>
+          <t>int[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="B123" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NumbersAdded</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>add(new int[] {1, 2}, 3).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D123" s="10" t="inlineStr">
+        <is>
+          <t>int[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="B124" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NumbersWithEmpty</t>
+        </is>
+      </c>
+      <c r="C124" s="5" t="inlineStr">
+        <is>
+          <t>add(new int[] {1, 2}, (Integer) null).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D124" s="10" t="inlineStr">
+        <is>
+          <t>Integer[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="B125" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NumbersWithFraction</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>add(new int[] {1, 2}, 2.5).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D125" s="10" t="inlineStr">
+        <is>
+          <t>double[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="B126" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$FractionAdded</t>
+        </is>
+      </c>
+      <c r="C126" s="5" t="inlineStr">
+        <is>
+          <t>add(new int[] {1, 2}, 2.5)</t>
+        </is>
+      </c>
+      <c r="D126" s="10" t="inlineStr">
+        <is>
+          <t>1, 2, 2.5</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1781,12 +2071,12 @@
     <mergeCell ref="B47:C47"/>
     <mergeCell ref="B78:C78"/>
     <mergeCell ref="B6:I6"/>
-    <mergeCell ref="B99:D99"/>
     <mergeCell ref="B89:C89"/>
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="B76:I76"/>
     <mergeCell ref="B62:D62"/>
     <mergeCell ref="B45:I45"/>
+    <mergeCell ref="B109:D109"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B82:C82"/>
     <mergeCell ref="B4:I4"/>
@@ -1802,7 +2092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I50"/>
+  <dimension ref="B2:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -1872,506 +2162,531 @@
     <row r="10">
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>RemoveMissingValue</t>
+          <t>RemoveAtFromMissing</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>= removeElement(new Integer[] {1, 2, 3}, 5)</t>
+          <t>= remove((Integer[]) null, 0)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>RemoveEmptyValue</t>
+          <t>RemoveMissingValue</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>= removeElement(new Integer[] {1, null, 3}, (Integer) null)</t>
+          <t>= removeElement(new Integer[] {1, 2, 3}, 5)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>RemoveOneOfTwo</t>
+          <t>RemoveEmptyValue</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>= removeElement(new int[] {1, 2, 2}, 2)</t>
+          <t>= removeElement(new Integer[] {1, null, 3}, (Integer) null)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>RemoveFromMissing</t>
+          <t>RemoveOneOfTwo</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>= removeElement((Integer[]) null, 5)</t>
+          <t>= removeElement(new int[] {1, 2, 2}, 2)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>RemoveNullValues</t>
+          <t>RemoveFromMissing</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>= removeNulls(1, null, 3)</t>
+          <t>= removeElement((Integer[]) null, 5)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>OnlyNulls</t>
+          <t>RemoveNullValues</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>= length(removeNulls(new Integer[] {null, null}))</t>
+          <t>= removeNulls(1, null, 3)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="6" t="inlineStr">
         <is>
+          <t>OnlyNulls</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>= length(removeNulls(new Integer[] {null, null}))</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="6" t="inlineStr">
+        <is>
           <t>RemoveNullsMissing</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>= removeNulls((Integer[]) null)</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="3" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Test RemoveExamples RemoveExamplesTest</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n"/>
-      <c r="D18" s="4" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$RemoveFirst</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>remove(new Integer[] {10, 20, 30}, 0)</t>
-        </is>
-      </c>
-      <c r="D19" s="10" t="inlineStr">
-        <is>
-          <t>20, 30</t>
-        </is>
-      </c>
+      <c r="C19" s="8" t="n"/>
+      <c r="D19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>_res_.$RemoveLast</t>
+          <t>_res_.$RemoveFirst</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>remove(new int[] {10, 20, 30}, 2)</t>
+          <t>remove(new Integer[] {10, 20, 30}, 0)</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>10, 20</t>
+          <t>20, 30</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>_res_.$RemoveMissingValue</t>
+          <t>_res_.$RemoveLast</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>removeElement(new Integer[] {1, 2, 3}, 5)</t>
+          <t>remove(new int[] {10, 20, 30}, 2)</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>1, 2, 3</t>
+          <t>10, 20</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>_res_.$RemoveEmptyValue</t>
+          <t>_res_.$RemoveAtFromMissing</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>removeElement(new Integer[] {1, null, 3}, (Integer) null)</t>
-        </is>
-      </c>
-      <c r="D22" s="10" t="inlineStr">
-        <is>
-          <t>1, 3</t>
-        </is>
-      </c>
+          <t>remove((Integer[]) null, 0)</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="n"/>
     </row>
     <row r="23">
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>_res_.$RemoveOneOfTwo</t>
+          <t>_res_.$RemoveMissingValue</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>removeElement(new int[] {1, 2, 2}, 2)</t>
+          <t>removeElement(new Integer[] {1, 2, 3}, 5)</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>1, 2</t>
+          <t>1, 2, 3</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>_res_.$RemoveFromMissing</t>
+          <t>_res_.$RemoveEmptyValue</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>removeElement((Integer[]) null, 5)</t>
-        </is>
-      </c>
-      <c r="D24" s="10" t="n"/>
+          <t>removeElement(new Integer[] {1, null, 3}, (Integer) null)</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>1, 3</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>_res_.$RemoveNullValues</t>
+          <t>_res_.$RemoveOneOfTwo</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>removeNulls(1, null, 3)</t>
+          <t>removeElement(new int[] {1, 2, 2}, 2)</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>1, 3</t>
+          <t>1, 2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>_res_.$OnlyNulls</t>
+          <t>_res_.$RemoveFromMissing</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>length(removeNulls(new Integer[] {null, null}))</t>
-        </is>
-      </c>
-      <c r="D26" s="10" t="n">
-        <v>0</v>
-      </c>
+          <t>removeElement((Integer[]) null, 5)</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="n"/>
     </row>
     <row r="27">
       <c r="B27" s="9" t="inlineStr">
         <is>
+          <t>_res_.$RemoveNullValues</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>removeNulls(1, null, 3)</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>1, 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$OnlyNulls</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>length(removeNulls(new Integer[] {null, null}))</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="9" t="inlineStr">
+        <is>
           <t>_res_.$RemoveNullsMissing</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>removeNulls((Integer[]) null)</t>
         </is>
       </c>
-      <c r="D27" s="10" t="n"/>
-    </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="B29" s="2" t="inlineStr">
+      <c r="D29" s="10" t="n"/>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>slice(array, start) and slice(array, start, end) copy the elements from the start position up to, but not including, the end position. A negative position counts from the end: -1 is the last element. Positions beyond the array are cut to its borders, so the result can be empty.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="3" t="inlineStr">
+    <row r="33">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>Spreadsheet SpreadsheetResult SliceExamples()</t>
         </is>
       </c>
-      <c r="C31" s="4" t="n"/>
-    </row>
-    <row r="32">
-      <c r="B32" s="5" t="inlineStr">
+      <c r="C33" s="4" t="n"/>
+    </row>
+    <row r="34">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>LastTwo</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>= slice(new Integer[] {1, 2, 3, 4, 5}, -2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="6" t="inlineStr">
-        <is>
-          <t>WithoutLast</t>
-        </is>
-      </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>= slice(new Integer[] {1, 2, 3, 4, 5}, 1, -1)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>FromEnd</t>
+          <t>LastTwo</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>= slice(new Integer[] {1, 2, 3, 4, 5}, -3, -1)</t>
+          <t>= slice(new Integer[] {1, 2, 3, 4, 5}, -2)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>StartTooFarBack</t>
+          <t>WithoutLast</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>= slice(new Integer[] {1, 2, 3, 4, 5}, -9)</t>
+          <t>= slice(new Integer[] {1, 2, 3, 4, 5}, 1, -1)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>EndTooFar</t>
+          <t>FromEnd</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>= slice(new Integer[] {1, 2, 3, 4, 5}, 2, 99)</t>
+          <t>= slice(new Integer[] {1, 2, 3, 4, 5}, -3, -1)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>StartAtLength</t>
+          <t>StartTooFarBack</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>= length(slice(new Integer[] {1, 2, 3, 4, 5}, 5))</t>
+          <t>= slice(new Integer[] {1, 2, 3, 4, 5}, -9)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>StartAfterEnd</t>
+          <t>EndTooFar</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>= length(slice(new Integer[] {1, 2, 3, 4, 5}, 3, 1))</t>
+          <t>= slice(new Integer[] {1, 2, 3, 4, 5}, 2, 99)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="6" t="inlineStr">
         <is>
+          <t>StartAtLength</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>= length(slice(new Integer[] {1, 2, 3, 4, 5}, 5))</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>StartAfterEnd</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>= length(slice(new Integer[] {1, 2, 3, 4, 5}, 3, 1))</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="6" t="inlineStr">
+        <is>
           <t>MissingArray</t>
         </is>
       </c>
-      <c r="C40" s="7" t="inlineStr">
+      <c r="C42" s="7" t="inlineStr">
         <is>
           <t>= slice((Integer[]) null, 2)</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="B42" s="3" t="inlineStr">
+    <row r="44">
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>Test SliceExamples SliceExamplesTest</t>
         </is>
       </c>
-      <c r="C42" s="8" t="n"/>
-      <c r="D42" s="4" t="n"/>
-    </row>
-    <row r="43">
-      <c r="B43" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$LastTwo</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>slice(new Integer[] {1, 2, 3, 4, 5}, -2)</t>
-        </is>
-      </c>
-      <c r="D43" s="10" t="inlineStr">
-        <is>
-          <t>4, 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$WithoutLast</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>slice(new Integer[] {1, 2, 3, 4, 5}, 1, -1)</t>
-        </is>
-      </c>
-      <c r="D44" s="10" t="inlineStr">
-        <is>
-          <t>2, 3, 4</t>
-        </is>
-      </c>
+      <c r="C44" s="8" t="n"/>
+      <c r="D44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>_res_.$FromEnd</t>
+          <t>_res_.$LastTwo</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>slice(new Integer[] {1, 2, 3, 4, 5}, -3, -1)</t>
+          <t>slice(new Integer[] {1, 2, 3, 4, 5}, -2)</t>
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>3, 4</t>
+          <t>4, 5</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>_res_.$StartTooFarBack</t>
+          <t>_res_.$WithoutLast</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>slice(new Integer[] {1, 2, 3, 4, 5}, -9)</t>
+          <t>slice(new Integer[] {1, 2, 3, 4, 5}, 1, -1)</t>
         </is>
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t>1, 2, 3, 4, 5</t>
+          <t>2, 3, 4</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>_res_.$EndTooFar</t>
+          <t>_res_.$FromEnd</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>slice(new Integer[] {1, 2, 3, 4, 5}, 2, 99)</t>
+          <t>slice(new Integer[] {1, 2, 3, 4, 5}, -3, -1)</t>
         </is>
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>3, 4, 5</t>
+          <t>3, 4</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>_res_.$StartAtLength</t>
+          <t>_res_.$StartTooFarBack</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>length(slice(new Integer[] {1, 2, 3, 4, 5}, 5))</t>
-        </is>
-      </c>
-      <c r="D48" s="10" t="n">
-        <v>0</v>
+          <t>slice(new Integer[] {1, 2, 3, 4, 5}, -9)</t>
+        </is>
+      </c>
+      <c r="D48" s="10" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
       </c>
     </row>
     <row r="49">
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>_res_.$StartAfterEnd</t>
+          <t>_res_.$EndTooFar</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>length(slice(new Integer[] {1, 2, 3, 4, 5}, 3, 1))</t>
-        </is>
-      </c>
-      <c r="D49" s="10" t="n">
-        <v>0</v>
+          <t>slice(new Integer[] {1, 2, 3, 4, 5}, 2, 99)</t>
+        </is>
+      </c>
+      <c r="D49" s="10" t="inlineStr">
+        <is>
+          <t>3, 4, 5</t>
+        </is>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="9" t="inlineStr">
         <is>
+          <t>_res_.$StartAtLength</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>length(slice(new Integer[] {1, 2, 3, 4, 5}, 5))</t>
+        </is>
+      </c>
+      <c r="D50" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$StartAfterEnd</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>length(slice(new Integer[] {1, 2, 3, 4, 5}, 3, 1))</t>
+        </is>
+      </c>
+      <c r="D51" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="9" t="inlineStr">
+        <is>
           <t>_res_.$MissingArray</t>
         </is>
       </c>
-      <c r="C50" s="5" t="inlineStr">
+      <c r="C52" s="5" t="inlineStr">
         <is>
           <t>slice((Integer[]) null, 2)</t>
         </is>
       </c>
-      <c r="D50" s="10" t="n"/>
+      <c r="D52" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="B42:D42"/>
     <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="B44:D44"/>
     <mergeCell ref="B4:I4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
EPBDS-16837 Fix flatten failing on int[] and returning an empty array for null
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/7-Functions/ArrayFunctions.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/7-Functions/ArrayFunctions.xlsx
@@ -550,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I126"/>
+  <dimension ref="B2:I132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -771,79 +771,69 @@
     <row r="24">
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Intersection</t>
+          <t>FlattenNumbers</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>= intersection(new String[] {"a", "b", "c"}, new String[] {"b", "c", "d"})</t>
+          <t>= flatten(new int[][] {{1, 2}, {3}})</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="6" t="inlineStr">
         <is>
+          <t>FlattenMissing</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>= flatten((int[]) null)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Intersection</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>= intersection(new String[] {"a", "b", "c"}, new String[] {"b", "c", "d"})</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="6" t="inlineStr">
+        <is>
           <t>Concatenate</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>= concatenate(new String[] {"a", "b"})</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="3" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Test BuildArrays BuildArraysTest</t>
         </is>
       </c>
-      <c r="C27" s="8" t="n"/>
-      <c r="D27" s="4" t="n"/>
-    </row>
-    <row r="28">
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$Add</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>add(new Integer[] {1, 2}, 3)</t>
-        </is>
-      </c>
-      <c r="D28" s="10" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$AddSeveral</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>add(new Integer[] {1, 2}, 3, 4)</t>
-        </is>
-      </c>
-      <c r="D29" s="10" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>_res_.$AddArrays</t>
+          <t>_res_.$Add</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>add(new Integer[] {1}, new Integer[] {2, 3})</t>
+          <t>add(new Integer[] {1, 2}, 3)</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
@@ -855,182 +845,182 @@
     <row r="31">
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>_res_.$AddAll</t>
+          <t>_res_.$AddSeveral</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>addAll(new Integer[] {1}, new Integer[] {2, 3})</t>
+          <t>add(new Integer[] {1, 2}, 3, 4)</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>1, 2, 3</t>
+          <t>1, 2, 3, 4</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>_res_.$Insert</t>
+          <t>_res_.$AddArrays</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>addElement(new String[] {"a", "c"}, 1, "b")</t>
+          <t>add(new Integer[] {1}, new Integer[] {2, 3})</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>a, b, c</t>
+          <t>1, 2, 3</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>_res_.$InsertArray</t>
+          <t>_res_.$AddAll</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>addElement(new String[] {"a", "d"}, 1, new String[] {"b", "c"})</t>
+          <t>addAll(new Integer[] {1}, new Integer[] {2, 3})</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>a, b, c, d</t>
+          <t>1, 2, 3</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>_res_.$RemoveAt</t>
+          <t>_res_.$Insert</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>remove(new Integer[] {10, 20, 30}, 1)</t>
+          <t>addElement(new String[] {"a", "c"}, 1, "b")</t>
         </is>
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t>10, 30</t>
+          <t>a, b, c</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>_res_.$RemoveFirstMatch</t>
+          <t>_res_.$InsertArray</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>removeElement(new String[] {"a", "b", "a"}, "a")</t>
+          <t>addElement(new String[] {"a", "d"}, 1, new String[] {"b", "c"})</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>b, a</t>
+          <t>a, b, c, d</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>_res_.$RemoveNulls</t>
+          <t>_res_.$RemoveAt</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>removeNulls(new String[] {"a", null, "b"})</t>
+          <t>remove(new Integer[] {10, 20, 30}, 1)</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>a, b</t>
+          <t>10, 30</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>_res_.$Slice</t>
+          <t>_res_.$RemoveFirstMatch</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>slice(new Integer[] {1, 2, 3, 4, 5}, 1, 3)</t>
+          <t>removeElement(new String[] {"a", "b", "a"}, "a")</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>2, 3</t>
+          <t>b, a</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>_res_.$SliceToEnd</t>
+          <t>_res_.$RemoveNulls</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>slice(new Integer[] {1, 2, 3, 4, 5}, 2)</t>
+          <t>removeNulls(new String[] {"a", null, "b"})</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>3, 4, 5</t>
+          <t>a, b</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>_res_.$Sort</t>
+          <t>_res_.$Slice</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>sort(new Integer[] {3, 1, 2})</t>
+          <t>slice(new Integer[] {1, 2, 3, 4, 5}, 1, 3)</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>1, 2, 3</t>
+          <t>2, 3</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>_res_.$SortText</t>
+          <t>_res_.$SliceToEnd</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>sort(new String[] {"pear", "Apple", "fig"})</t>
+          <t>slice(new Integer[] {1, 2, 3, 4, 5}, 2)</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>Apple, fig, pear</t>
+          <t>3, 4, 5</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="9" t="inlineStr">
         <is>
-          <t>_res_.$Flatten</t>
+          <t>_res_.$Sort</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>flatten(new Integer[][] {{1, 2}, {3}})</t>
+          <t>sort(new Integer[] {3, 1, 2})</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
@@ -1042,954 +1032,945 @@
     <row r="42">
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>_res_.$Intersection</t>
+          <t>_res_.$SortText</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>intersection(new String[] {"a", "b", "c"}, new String[] {"b", "c", "d"})</t>
+          <t>sort(new String[] {"pear", "Apple", "fig"})</t>
         </is>
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>b, c</t>
+          <t>Apple, fig, pear</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="9" t="inlineStr">
         <is>
+          <t>_res_.$Flatten</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>flatten(new Integer[][] {{1, 2}, {3}})</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$FlattenNumbers</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>flatten(new int[][] {{1, 2}, {3}})</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$FlattenMissing</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>flatten((int[]) null)</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="n"/>
+    </row>
+    <row r="46">
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Intersection</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>intersection(new String[] {"a", "b", "c"}, new String[] {"b", "c", "d"})</t>
+        </is>
+      </c>
+      <c r="D46" s="10" t="inlineStr">
+        <is>
+          <t>b, c</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="9" t="inlineStr">
+        <is>
           <t>_res_.$Concatenate</t>
         </is>
       </c>
-      <c r="C43" s="5" t="inlineStr">
+      <c r="C47" s="5" t="inlineStr">
         <is>
           <t>concatenate(new String[] {"a", "b"})</t>
         </is>
       </c>
-      <c r="D43" s="10" t="inlineStr">
+      <c r="D47" s="10" t="inlineStr">
         <is>
           <t>ab</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="30" customHeight="1">
-      <c r="B45" s="2" t="inlineStr">
+    <row r="49" ht="30" customHeight="1">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>add also builds an array from single values, and works with an empty array or element. An empty array counts as an array without elements; an empty element is added as an empty value. addElement inserts at any position from 0 to the length of the array.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="B47" s="3" t="inlineStr">
+    <row r="51">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>Spreadsheet SpreadsheetResult AddEdgeCases()</t>
         </is>
       </c>
-      <c r="C47" s="4" t="n"/>
-    </row>
-    <row r="48">
-      <c r="B48" s="5" t="inlineStr">
+      <c r="C51" s="4" t="n"/>
+    </row>
+    <row r="52">
+      <c r="B52" s="5" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="C52" s="5" t="inlineStr">
         <is>
           <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="B49" s="6" t="inlineStr">
-        <is>
-          <t>FromValues</t>
-        </is>
-      </c>
-      <c r="C49" s="7" t="inlineStr">
-        <is>
-          <t>= add(1, 2, 3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="B50" s="6" t="inlineStr">
-        <is>
-          <t>FromTexts</t>
-        </is>
-      </c>
-      <c r="C50" s="7" t="inlineStr">
-        <is>
-          <t>= add("a", "b")</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="B51" s="6" t="inlineStr">
-        <is>
-          <t>ToEmptyArray</t>
-        </is>
-      </c>
-      <c r="C51" s="7" t="inlineStr">
-        <is>
-          <t>= add((Integer[]) null, 5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="B52" s="6" t="inlineStr">
-        <is>
-          <t>EmptyElement</t>
-        </is>
-      </c>
-      <c r="C52" s="7" t="inlineStr">
-        <is>
-          <t>= length(add(new Integer[] {1, 2}, (Integer) null))</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>EmptyElementValue</t>
+          <t>FromValues</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>= add(new Integer[] {1, 2}, (Integer) null)[2]</t>
+          <t>= add(1, 2, 3)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>EmptySecondArray</t>
+          <t>FromTexts</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>= add(new Integer[] {1, 2}, (Integer[]) null)</t>
+          <t>= add("a", "b")</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>NumbersArray</t>
+          <t>ToEmptyArray</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>= add(new int[] {1, 2}, new int[] {3, 4})</t>
+          <t>= add((Integer[]) null, 5)</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>Dates</t>
+          <t>EmptyElement</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>= length(add(new Date[] {Date(2024, 1, 1)}, Date(2024, 2, 1)))</t>
+          <t>= length(add(new Integer[] {1, 2}, (Integer) null))</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>InsertFirst</t>
+          <t>EmptyElementValue</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>= addElement(new Integer[] {1, 2}, 0, 0)</t>
+          <t>= add(new Integer[] {1, 2}, (Integer) null)[2]</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>InsertLast</t>
+          <t>EmptySecondArray</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>= addElement(new Integer[] {1, 2}, 2, 3)</t>
+          <t>= add(new Integer[] {1, 2}, (Integer[]) null)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>InsertIntoEmpty</t>
+          <t>NumbersArray</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>= addElement((Integer[]) null, 0, 5)</t>
+          <t>= add(new int[] {1, 2}, new int[] {3, 4})</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="B60" s="6" t="inlineStr">
         <is>
+          <t>Dates</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>= length(add(new Date[] {Date(2024, 1, 1)}, Date(2024, 2, 1)))</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>InsertFirst</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>= addElement(new Integer[] {1, 2}, 0, 0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>InsertLast</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>= addElement(new Integer[] {1, 2}, 2, 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>InsertIntoEmpty</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>= addElement((Integer[]) null, 0, 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="6" t="inlineStr">
+        <is>
           <t>InsertEmptyValue</t>
         </is>
       </c>
-      <c r="C60" s="7" t="inlineStr">
+      <c r="C64" s="7" t="inlineStr">
         <is>
           <t>= addElement(new Integer[] {1, 2}, 1, (Integer) null)[1]</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="B62" s="3" t="inlineStr">
+    <row r="66">
+      <c r="B66" s="3" t="inlineStr">
         <is>
           <t>Test AddEdgeCases AddEdgeCasesTest</t>
         </is>
       </c>
-      <c r="C62" s="8" t="n"/>
-      <c r="D62" s="4" t="n"/>
-    </row>
-    <row r="63">
-      <c r="B63" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$FromValues</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>add(1, 2, 3)</t>
-        </is>
-      </c>
-      <c r="D63" s="10" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="B64" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$FromTexts</t>
-        </is>
-      </c>
-      <c r="C64" s="5" t="inlineStr">
-        <is>
-          <t>add("a", "b")</t>
-        </is>
-      </c>
-      <c r="D64" s="10" t="inlineStr">
-        <is>
-          <t>a, b</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="B65" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$ToEmptyArray</t>
-        </is>
-      </c>
-      <c r="C65" s="5" t="inlineStr">
-        <is>
-          <t>add((Integer[]) null, 5)</t>
-        </is>
-      </c>
-      <c r="D65" s="10" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="B66" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$EmptyElement</t>
-        </is>
-      </c>
-      <c r="C66" s="5" t="inlineStr">
-        <is>
-          <t>length(add(new Integer[] {1, 2}, (Integer) null))</t>
-        </is>
-      </c>
-      <c r="D66" s="10" t="n">
-        <v>3</v>
-      </c>
+      <c r="C66" s="8" t="n"/>
+      <c r="D66" s="4" t="n"/>
     </row>
     <row r="67">
       <c r="B67" s="9" t="inlineStr">
         <is>
-          <t>_res_.$EmptyElementValue</t>
+          <t>_res_.$FromValues</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>add(new Integer[] {1, 2}, (Integer) null)[2]</t>
-        </is>
-      </c>
-      <c r="D67" s="10" t="n"/>
+          <t>add(1, 2, 3)</t>
+        </is>
+      </c>
+      <c r="D67" s="10" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="B68" s="9" t="inlineStr">
         <is>
-          <t>_res_.$EmptySecondArray</t>
+          <t>_res_.$FromTexts</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>add(new Integer[] {1, 2}, (Integer[]) null)</t>
+          <t>add("a", "b")</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t>1, 2</t>
+          <t>a, b</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="B69" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NumbersArray</t>
+          <t>_res_.$ToEmptyArray</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>add(new int[] {1, 2}, new int[] {3, 4})</t>
+          <t>add((Integer[]) null, 5)</t>
         </is>
       </c>
       <c r="D69" s="10" t="inlineStr">
         <is>
-          <t>1, 2, 3, 4</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="B70" s="9" t="inlineStr">
         <is>
-          <t>_res_.$Dates</t>
+          <t>_res_.$EmptyElement</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>length(add(new Date[] {Date(2024, 1, 1)}, Date(2024, 2, 1)))</t>
+          <t>length(add(new Integer[] {1, 2}, (Integer) null))</t>
         </is>
       </c>
       <c r="D70" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="71">
       <c r="B71" s="9" t="inlineStr">
         <is>
-          <t>_res_.$InsertFirst</t>
+          <t>_res_.$EmptyElementValue</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>addElement(new Integer[] {1, 2}, 0, 0)</t>
-        </is>
-      </c>
-      <c r="D71" s="10" t="inlineStr">
-        <is>
-          <t>0, 1, 2</t>
-        </is>
-      </c>
+          <t>add(new Integer[] {1, 2}, (Integer) null)[2]</t>
+        </is>
+      </c>
+      <c r="D71" s="10" t="n"/>
     </row>
     <row r="72">
       <c r="B72" s="9" t="inlineStr">
         <is>
-          <t>_res_.$InsertLast</t>
+          <t>_res_.$EmptySecondArray</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>addElement(new Integer[] {1, 2}, 2, 3)</t>
+          <t>add(new Integer[] {1, 2}, (Integer[]) null)</t>
         </is>
       </c>
       <c r="D72" s="10" t="inlineStr">
         <is>
-          <t>1, 2, 3</t>
+          <t>1, 2</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="B73" s="9" t="inlineStr">
         <is>
-          <t>_res_.$InsertIntoEmpty</t>
+          <t>_res_.$NumbersArray</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>addElement((Integer[]) null, 0, 5)</t>
+          <t>add(new int[] {1, 2}, new int[] {3, 4})</t>
         </is>
       </c>
       <c r="D73" s="10" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1, 2, 3, 4</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="B74" s="9" t="inlineStr">
         <is>
+          <t>_res_.$Dates</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>length(add(new Date[] {Date(2024, 1, 1)}, Date(2024, 2, 1)))</t>
+        </is>
+      </c>
+      <c r="D74" s="10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$InsertFirst</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>addElement(new Integer[] {1, 2}, 0, 0)</t>
+        </is>
+      </c>
+      <c r="D75" s="10" t="inlineStr">
+        <is>
+          <t>0, 1, 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$InsertLast</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>addElement(new Integer[] {1, 2}, 2, 3)</t>
+        </is>
+      </c>
+      <c r="D76" s="10" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$InsertIntoEmpty</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>addElement((Integer[]) null, 0, 5)</t>
+        </is>
+      </c>
+      <c r="D77" s="10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="9" t="inlineStr">
+        <is>
           <t>_res_.$InsertEmptyValue</t>
         </is>
       </c>
-      <c r="C74" s="5" t="inlineStr">
+      <c r="C78" s="5" t="inlineStr">
         <is>
           <t>addElement(new Integer[] {1, 2}, 1, (Integer) null)[1]</t>
         </is>
       </c>
-      <c r="D74" s="10" t="n"/>
-    </row>
-    <row r="76" ht="30" customHeight="1">
-      <c r="B76" s="2" t="inlineStr">
+      <c r="D78" s="10" t="n"/>
+    </row>
+    <row r="80" ht="30" customHeight="1">
+      <c r="B80" s="2" t="inlineStr">
         <is>
           <t>The functions keep the element type: applied to an array of a datatype, they return an array of the same datatype, so a field of an element is read directly without a cast. A primitive array, such as int[], stays int[]. add, addAll and addElement change the type only to fit an added element: an Integer gives Integer[], so that the element can be empty, and a fraction gives double[].</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="B78" s="3" t="inlineStr">
-        <is>
-          <t>Datatype Country</t>
-        </is>
-      </c>
-      <c r="C78" s="4" t="n"/>
-    </row>
-    <row r="79">
-      <c r="B79" s="6" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="C79" s="6" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="B80" s="6" t="inlineStr">
-        <is>
-          <t>Integer</t>
-        </is>
-      </c>
-      <c r="C80" s="6" t="inlineStr">
-        <is>
-          <t>code</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="B82" s="3" t="inlineStr">
         <is>
+          <t>Datatype Country</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="n"/>
+    </row>
+    <row r="83">
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" s="3" t="inlineStr">
+        <is>
           <t>Data Country countries</t>
         </is>
       </c>
-      <c r="C82" s="4" t="n"/>
-    </row>
-    <row r="83">
-      <c r="B83" s="9" t="inlineStr">
+      <c r="C86" s="4" t="n"/>
+    </row>
+    <row r="87">
+      <c r="B87" s="9" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C83" s="9" t="inlineStr">
+      <c r="C87" s="9" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="B84" s="5" t="inlineStr">
+    <row r="88">
+      <c r="B88" s="5" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C84" s="5" t="inlineStr">
+      <c r="C88" s="5" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="B85" s="6" t="inlineStr">
+    <row r="89">
+      <c r="B89" s="6" t="inlineStr">
         <is>
           <t>Austria</t>
         </is>
       </c>
-      <c r="C85" s="6" t="n">
+      <c r="C89" s="6" t="n">
         <v>43</v>
       </c>
     </row>
-    <row r="86">
-      <c r="B86" s="6" t="inlineStr">
+    <row r="90">
+      <c r="B90" s="6" t="inlineStr">
         <is>
           <t>Brazil</t>
         </is>
       </c>
-      <c r="C86" s="6" t="n">
+      <c r="C90" s="6" t="n">
         <v>55</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="B87" s="6" t="inlineStr">
-        <is>
-          <t>Chile</t>
-        </is>
-      </c>
-      <c r="C87" s="6" t="n">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="B89" s="3" t="inlineStr">
-        <is>
-          <t>Spreadsheet SpreadsheetResult TypedResults()</t>
-        </is>
-      </c>
-      <c r="C89" s="4" t="n"/>
-    </row>
-    <row r="90">
-      <c r="B90" s="5" t="inlineStr">
-        <is>
-          <t>Step</t>
-        </is>
-      </c>
-      <c r="C90" s="5" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
       </c>
     </row>
     <row r="91">
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>Added</t>
-        </is>
-      </c>
-      <c r="C91" s="7" t="inlineStr">
-        <is>
-          <t>= add(countries, new Country(name = "Denmark"))[3].name</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="B92" s="6" t="inlineStr">
-        <is>
-          <t>AddedNames</t>
-        </is>
-      </c>
-      <c r="C92" s="7" t="inlineStr">
-        <is>
-          <t>= add(countries, new Country(name = "Denmark")).name</t>
-        </is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="C91" s="6" t="n">
+        <v>56</v>
       </c>
     </row>
     <row r="93">
-      <c r="B93" s="6" t="inlineStr">
-        <is>
-          <t>AddedAll</t>
-        </is>
-      </c>
-      <c r="C93" s="7" t="inlineStr">
-        <is>
-          <t>= addAll(countries, countries)[4].name</t>
-        </is>
-      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>Spreadsheet SpreadsheetResult TypedResults()</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="n"/>
     </row>
     <row r="94">
-      <c r="B94" s="6" t="inlineStr">
-        <is>
-          <t>Inserted</t>
-        </is>
-      </c>
-      <c r="C94" s="7" t="inlineStr">
-        <is>
-          <t>= addElement(countries, 1, new Country(name = "Denmark"))[1].name</t>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>Removed</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>= remove(countries, 0)[0].name</t>
+          <t>= add(countries, new Country(name = "Denmark"))[3].name</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>RemovedElement</t>
+          <t>AddedNames</t>
         </is>
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>= removeElement(countries, countries[1]).name</t>
+          <t>= add(countries, new Country(name = "Denmark")).name</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>WithoutNulls</t>
+          <t>AddedAll</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>= removeNulls(new Country[] {null, countries[2]})[0].code</t>
+          <t>= addAll(countries, countries)[4].name</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="B98" s="6" t="inlineStr">
         <is>
-          <t>NumbersSorted</t>
+          <t>Inserted</t>
         </is>
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>= sort(new int[] {3, 1, 2}).getClass().getSimpleName()</t>
+          <t>= addElement(countries, 1, new Country(name = "Denmark"))[1].name</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>NumbersSliced</t>
+          <t>Removed</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>= slice(new int[] {1, 2, 3}, 1).getClass().getSimpleName()</t>
+          <t>= remove(countries, 0)[0].name</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="B100" s="6" t="inlineStr">
         <is>
-          <t>NumbersRemoved</t>
+          <t>RemovedElement</t>
         </is>
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>= remove(new int[] {1, 2}, 0).getClass().getSimpleName()</t>
+          <t>= removeElement(countries, countries[1]).name</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="B101" s="6" t="inlineStr">
         <is>
-          <t>NumbersRemovedElement</t>
+          <t>WithoutNulls</t>
         </is>
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>= removeElement(new int[] {1, 2}, 1).getClass().getSimpleName()</t>
+          <t>= removeNulls(new Country[] {null, countries[2]})[0].code</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="B102" s="6" t="inlineStr">
         <is>
-          <t>NumbersWithoutNulls</t>
+          <t>NumbersSorted</t>
         </is>
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>= removeNulls(new int[] {1, 2}).getClass().getSimpleName()</t>
+          <t>= sort(new int[] {3, 1, 2}).getClass().getSimpleName()</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="B103" s="6" t="inlineStr">
         <is>
-          <t>NumbersInserted</t>
+          <t>NumbersSliced</t>
         </is>
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>= addElement(new int[] {1, 2}, 1, 5).getClass().getSimpleName()</t>
+          <t>= slice(new int[] {1, 2, 3}, 1).getClass().getSimpleName()</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="B104" s="6" t="inlineStr">
         <is>
-          <t>NumbersAdded</t>
+          <t>NumbersRemoved</t>
         </is>
       </c>
       <c r="C104" s="7" t="inlineStr">
         <is>
-          <t>= add(new int[] {1, 2}, 3).getClass().getSimpleName()</t>
+          <t>= remove(new int[] {1, 2}, 0).getClass().getSimpleName()</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="B105" s="6" t="inlineStr">
         <is>
-          <t>NumbersWithEmpty</t>
+          <t>NumbersRemovedElement</t>
         </is>
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>= add(new int[] {1, 2}, (Integer) null).getClass().getSimpleName()</t>
+          <t>= removeElement(new int[] {1, 2}, 1).getClass().getSimpleName()</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="B106" s="6" t="inlineStr">
         <is>
-          <t>NumbersWithFraction</t>
+          <t>NumbersWithoutNulls</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
         <is>
-          <t>= add(new int[] {1, 2}, 2.5).getClass().getSimpleName()</t>
+          <t>= removeNulls(new int[] {1, 2}).getClass().getSimpleName()</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="B107" s="6" t="inlineStr">
         <is>
+          <t>NumbersInserted</t>
+        </is>
+      </c>
+      <c r="C107" s="7" t="inlineStr">
+        <is>
+          <t>= addElement(new int[] {1, 2}, 1, 5).getClass().getSimpleName()</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="B108" s="6" t="inlineStr">
+        <is>
+          <t>NumbersAdded</t>
+        </is>
+      </c>
+      <c r="C108" s="7" t="inlineStr">
+        <is>
+          <t>= add(new int[] {1, 2}, 3).getClass().getSimpleName()</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="B109" s="6" t="inlineStr">
+        <is>
+          <t>NumbersWithEmpty</t>
+        </is>
+      </c>
+      <c r="C109" s="7" t="inlineStr">
+        <is>
+          <t>= add(new int[] {1, 2}, (Integer) null).getClass().getSimpleName()</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="B110" s="6" t="inlineStr">
+        <is>
+          <t>NumbersWithFraction</t>
+        </is>
+      </c>
+      <c r="C110" s="7" t="inlineStr">
+        <is>
+          <t>= add(new int[] {1, 2}, 2.5).getClass().getSimpleName()</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="B111" s="6" t="inlineStr">
+        <is>
           <t>FractionAdded</t>
         </is>
       </c>
-      <c r="C107" s="7" t="inlineStr">
+      <c r="C111" s="7" t="inlineStr">
         <is>
           <t>= add(new int[] {1, 2}, 2.5)</t>
         </is>
       </c>
     </row>
-    <row r="109">
-      <c r="B109" s="3" t="inlineStr">
+    <row r="112">
+      <c r="B112" s="6" t="inlineStr">
+        <is>
+          <t>NumbersFlattened</t>
+        </is>
+      </c>
+      <c r="C112" s="7" t="inlineStr">
+        <is>
+          <t>= flatten(new int[][] {{1, 2}, {3}}).getClass().getSimpleName()</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" s="3" t="inlineStr">
         <is>
           <t>Test TypedResults TypedResultsTest</t>
         </is>
       </c>
-      <c r="C109" s="8" t="n"/>
-      <c r="D109" s="4" t="n"/>
-    </row>
-    <row r="110">
-      <c r="B110" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$Added</t>
-        </is>
-      </c>
-      <c r="C110" s="5" t="inlineStr">
-        <is>
-          <t>add(countries, new Country(name = "Denmark"))[3].name</t>
-        </is>
-      </c>
-      <c r="D110" s="10" t="inlineStr">
-        <is>
-          <t>Denmark</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="B111" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$AddedNames</t>
-        </is>
-      </c>
-      <c r="C111" s="5" t="inlineStr">
-        <is>
-          <t>add(countries, new Country(name = "Denmark")).name</t>
-        </is>
-      </c>
-      <c r="D111" s="10" t="inlineStr">
-        <is>
-          <t>Austria, Brazil, Chile, Denmark</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="B112" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$AddedAll</t>
-        </is>
-      </c>
-      <c r="C112" s="5" t="inlineStr">
-        <is>
-          <t>addAll(countries, countries)[4].name</t>
-        </is>
-      </c>
-      <c r="D112" s="10" t="inlineStr">
-        <is>
-          <t>Brazil</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="B113" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$Inserted</t>
-        </is>
-      </c>
-      <c r="C113" s="5" t="inlineStr">
-        <is>
-          <t>addElement(countries, 1, new Country(name = "Denmark"))[1].name</t>
-        </is>
-      </c>
-      <c r="D113" s="10" t="inlineStr">
-        <is>
-          <t>Denmark</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="B114" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$Removed</t>
-        </is>
-      </c>
-      <c r="C114" s="5" t="inlineStr">
-        <is>
-          <t>remove(countries, 0)[0].name</t>
-        </is>
-      </c>
-      <c r="D114" s="10" t="inlineStr">
-        <is>
-          <t>Brazil</t>
-        </is>
-      </c>
+      <c r="C114" s="8" t="n"/>
+      <c r="D114" s="4" t="n"/>
     </row>
     <row r="115">
       <c r="B115" s="9" t="inlineStr">
         <is>
-          <t>_res_.$RemovedElement</t>
+          <t>_res_.$Added</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>removeElement(countries, countries[1]).name</t>
+          <t>add(countries, new Country(name = "Denmark"))[3].name</t>
         </is>
       </c>
       <c r="D115" s="10" t="inlineStr">
         <is>
-          <t>Austria, Chile</t>
+          <t>Denmark</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="B116" s="9" t="inlineStr">
         <is>
-          <t>_res_.$WithoutNulls</t>
+          <t>_res_.$AddedNames</t>
         </is>
       </c>
       <c r="C116" s="5" t="inlineStr">
         <is>
-          <t>removeNulls(new Country[] {null, countries[2]})[0].code</t>
-        </is>
-      </c>
-      <c r="D116" s="10" t="n">
-        <v>56</v>
+          <t>add(countries, new Country(name = "Denmark")).name</t>
+        </is>
+      </c>
+      <c r="D116" s="10" t="inlineStr">
+        <is>
+          <t>Austria, Brazil, Chile, Denmark</t>
+        </is>
       </c>
     </row>
     <row r="117">
       <c r="B117" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NumbersSorted</t>
+          <t>_res_.$AddedAll</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>sort(new int[] {3, 1, 2}).getClass().getSimpleName()</t>
+          <t>addAll(countries, countries)[4].name</t>
         </is>
       </c>
       <c r="D117" s="10" t="inlineStr">
         <is>
-          <t>int[]</t>
+          <t>Brazil</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="B118" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NumbersSliced</t>
+          <t>_res_.$Inserted</t>
         </is>
       </c>
       <c r="C118" s="5" t="inlineStr">
         <is>
-          <t>slice(new int[] {1, 2, 3}, 1).getClass().getSimpleName()</t>
+          <t>addElement(countries, 1, new Country(name = "Denmark"))[1].name</t>
         </is>
       </c>
       <c r="D118" s="10" t="inlineStr">
         <is>
-          <t>int[]</t>
+          <t>Denmark</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="B119" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NumbersRemoved</t>
+          <t>_res_.$Removed</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>remove(new int[] {1, 2}, 0).getClass().getSimpleName()</t>
+          <t>remove(countries, 0)[0].name</t>
         </is>
       </c>
       <c r="D119" s="10" t="inlineStr">
         <is>
-          <t>int[]</t>
+          <t>Brazil</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="B120" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NumbersRemovedElement</t>
+          <t>_res_.$RemovedElement</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
         <is>
-          <t>removeElement(new int[] {1, 2}, 1).getClass().getSimpleName()</t>
+          <t>removeElement(countries, countries[1]).name</t>
         </is>
       </c>
       <c r="D120" s="10" t="inlineStr">
         <is>
-          <t>int[]</t>
+          <t>Austria, Chile</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="B121" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NumbersWithoutNulls</t>
+          <t>_res_.$WithoutNulls</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>removeNulls(new int[] {1, 2}).getClass().getSimpleName()</t>
-        </is>
-      </c>
-      <c r="D121" s="10" t="inlineStr">
-        <is>
-          <t>int[]</t>
-        </is>
+          <t>removeNulls(new Country[] {null, countries[2]})[0].code</t>
+        </is>
+      </c>
+      <c r="D121" s="10" t="n">
+        <v>56</v>
       </c>
     </row>
     <row r="122">
       <c r="B122" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NumbersInserted</t>
+          <t>_res_.$NumbersSorted</t>
         </is>
       </c>
       <c r="C122" s="5" t="inlineStr">
         <is>
-          <t>addElement(new int[] {1, 2}, 1, 5).getClass().getSimpleName()</t>
+          <t>sort(new int[] {3, 1, 2}).getClass().getSimpleName()</t>
         </is>
       </c>
       <c r="D122" s="10" t="inlineStr">
@@ -2001,12 +1982,12 @@
     <row r="123">
       <c r="B123" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NumbersAdded</t>
+          <t>_res_.$NumbersSliced</t>
         </is>
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>add(new int[] {1, 2}, 3).getClass().getSimpleName()</t>
+          <t>slice(new int[] {1, 2, 3}, 1).getClass().getSimpleName()</t>
         </is>
       </c>
       <c r="D123" s="10" t="inlineStr">
@@ -2018,65 +1999,167 @@
     <row r="124">
       <c r="B124" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NumbersWithEmpty</t>
+          <t>_res_.$NumbersRemoved</t>
         </is>
       </c>
       <c r="C124" s="5" t="inlineStr">
         <is>
-          <t>add(new int[] {1, 2}, (Integer) null).getClass().getSimpleName()</t>
+          <t>remove(new int[] {1, 2}, 0).getClass().getSimpleName()</t>
         </is>
       </c>
       <c r="D124" s="10" t="inlineStr">
         <is>
-          <t>Integer[]</t>
+          <t>int[]</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="B125" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NumbersWithFraction</t>
+          <t>_res_.$NumbersRemovedElement</t>
         </is>
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>add(new int[] {1, 2}, 2.5).getClass().getSimpleName()</t>
+          <t>removeElement(new int[] {1, 2}, 1).getClass().getSimpleName()</t>
         </is>
       </c>
       <c r="D125" s="10" t="inlineStr">
         <is>
-          <t>double[]</t>
+          <t>int[]</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="B126" s="9" t="inlineStr">
         <is>
+          <t>_res_.$NumbersWithoutNulls</t>
+        </is>
+      </c>
+      <c r="C126" s="5" t="inlineStr">
+        <is>
+          <t>removeNulls(new int[] {1, 2}).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D126" s="10" t="inlineStr">
+        <is>
+          <t>int[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="B127" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NumbersInserted</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="inlineStr">
+        <is>
+          <t>addElement(new int[] {1, 2}, 1, 5).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D127" s="10" t="inlineStr">
+        <is>
+          <t>int[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="B128" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NumbersAdded</t>
+        </is>
+      </c>
+      <c r="C128" s="5" t="inlineStr">
+        <is>
+          <t>add(new int[] {1, 2}, 3).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D128" s="10" t="inlineStr">
+        <is>
+          <t>int[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="B129" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NumbersWithEmpty</t>
+        </is>
+      </c>
+      <c r="C129" s="5" t="inlineStr">
+        <is>
+          <t>add(new int[] {1, 2}, (Integer) null).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D129" s="10" t="inlineStr">
+        <is>
+          <t>Integer[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="B130" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NumbersWithFraction</t>
+        </is>
+      </c>
+      <c r="C130" s="5" t="inlineStr">
+        <is>
+          <t>add(new int[] {1, 2}, 2.5).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D130" s="10" t="inlineStr">
+        <is>
+          <t>double[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="B131" s="9" t="inlineStr">
+        <is>
           <t>_res_.$FractionAdded</t>
         </is>
       </c>
-      <c r="C126" s="5" t="inlineStr">
+      <c r="C131" s="5" t="inlineStr">
         <is>
           <t>add(new int[] {1, 2}, 2.5)</t>
         </is>
       </c>
-      <c r="D126" s="10" t="inlineStr">
+      <c r="D131" s="10" t="inlineStr">
         <is>
           <t>1, 2, 2.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="B132" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NumbersFlattened</t>
+        </is>
+      </c>
+      <c r="C132" s="5" t="inlineStr">
+        <is>
+          <t>flatten(new int[][] {{1, 2}, {3}}).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D132" s="10" t="inlineStr">
+        <is>
+          <t>int[]</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B78:C78"/>
+    <mergeCell ref="B114:D114"/>
+    <mergeCell ref="B93:C93"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B49:I49"/>
+    <mergeCell ref="B86:C86"/>
+    <mergeCell ref="B66:D66"/>
     <mergeCell ref="B6:I6"/>
-    <mergeCell ref="B89:C89"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="B76:I76"/>
-    <mergeCell ref="B62:D62"/>
-    <mergeCell ref="B45:I45"/>
-    <mergeCell ref="B109:D109"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="B80:I80"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B82:C82"/>
     <mergeCell ref="B4:I4"/>
@@ -2685,8 +2768,8 @@
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B44:D44"/>
     <mergeCell ref="B31:I31"/>
-    <mergeCell ref="B44:D44"/>
     <mergeCell ref="B4:I4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>